<commit_message>
Match Endr Quote Submission options to the recording; blank Legal Verification on row 4
All admin requirements received offers Accepted/No/Yes only, as shown in the
recording. 112333103001 opens with Legal Verification blank so the SOP's
"if not pre-populated" step is exercised from the dummy work list.
</commit_message>
<xml_diff>
--- a/worklist/Fee Switch-Off Calculations.xlsx
+++ b/worklist/Fee Switch-Off Calculations.xlsx
@@ -464,6 +464,9 @@
     <t>9011220195083</t>
   </si>
   <si>
+    <t>(blank)</t>
+  </si>
+  <si>
     <t>31/07/2026</t>
   </si>
   <si>
@@ -539,9 +542,6 @@
     <t>9107122197084</t>
   </si>
   <si>
-    <t>(blank)</t>
-  </si>
-  <si>
     <t>7504077586083</t>
   </si>
   <si>
@@ -680,7 +680,7 @@
     <t>Endr Quote Submission → Submit</t>
   </si>
   <si>
-    <t>Activate, verifier side</t>
+    <t>Activate (closed book)</t>
   </si>
   <si>
     <t>One full case</t>
@@ -3346,10 +3346,10 @@
         <v>0.863</v>
       </c>
       <c r="I7" s="23" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="J7" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K7" s="5" t="str">
         <f>IF(E7="MISMATCH","STOP: ID number does not match the work list",IF(F7="Yes","STOP: error 56000, an endorsement is already in progress",IF(H7=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="M7" s="5" t="str">
         <f>IF(LEFT(K7,7)&lt;&gt;"PROCEED","n/a",IF(I7="(blank)","Select Approved before Submit","Already Approved"))</f>
-        <v>Already Approved</v>
+        <v>Select Approved before Submit</v>
       </c>
       <c r="N7" s="18" t="str">
         <f>IF(LEFT(K7,7)="PROCEED",J7,"n/a")</f>
@@ -3376,10 +3376,10 @@
         <v>77</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E8" s="18" t="str">
         <f>IF(C8=D8,"MATCH","MISMATCH")</f>
@@ -3399,7 +3399,7 @@
         <v>144</v>
       </c>
       <c r="J8" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K8" s="5" t="str">
         <f>IF(E8="MISMATCH","STOP: ID number does not match the work list",IF(F8="Yes","STOP: error 56000, an endorsement is already in progress",IF(H8=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3426,10 +3426,10 @@
         <v>79</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E9" s="18" t="str">
         <f>IF(C9=D9,"MATCH","MISMATCH")</f>
@@ -3449,7 +3449,7 @@
         <v>144</v>
       </c>
       <c r="J9" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K9" s="5" t="str">
         <f>IF(E9="MISMATCH","STOP: ID number does not match the work list",IF(F9="Yes","STOP: error 56000, an endorsement is already in progress",IF(H9=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3476,10 +3476,10 @@
         <v>81</v>
       </c>
       <c r="C10" s="22" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D10" s="22" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E10" s="18" t="str">
         <f>IF(C10=D10,"MATCH","MISMATCH")</f>
@@ -3526,10 +3526,10 @@
         <v>83</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E11" s="18" t="str">
         <f>IF(C11=D11,"MATCH","MISMATCH")</f>
@@ -3576,10 +3576,10 @@
         <v>85</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E12" s="18" t="str">
         <f>IF(C12=D12,"MATCH","MISMATCH")</f>
@@ -3599,7 +3599,7 @@
         <v>144</v>
       </c>
       <c r="J12" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K12" s="5" t="str">
         <f>IF(E12="MISMATCH","STOP: ID number does not match the work list",IF(F12="Yes","STOP: error 56000, an endorsement is already in progress",IF(H12=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3626,10 +3626,10 @@
         <v>87</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E13" s="18" t="str">
         <f>IF(C13=D13,"MATCH","MISMATCH")</f>
@@ -3649,7 +3649,7 @@
         <v>144</v>
       </c>
       <c r="J13" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K13" s="5" t="str">
         <f>IF(E13="MISMATCH","STOP: ID number does not match the work list",IF(F13="Yes","STOP: error 56000, an endorsement is already in progress",IF(H13=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3676,10 +3676,10 @@
         <v>89</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E14" s="18" t="str">
         <f>IF(C14=D14,"MATCH","MISMATCH")</f>
@@ -3699,7 +3699,7 @@
         <v>144</v>
       </c>
       <c r="J14" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K14" s="5" t="str">
         <f>IF(E14="MISMATCH","STOP: ID number does not match the work list",IF(F14="Yes","STOP: error 56000, an endorsement is already in progress",IF(H14=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3726,10 +3726,10 @@
         <v>91</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="E15" s="18" t="str">
         <f>IF(C15=D15,"MATCH","MISMATCH")</f>
@@ -3776,10 +3776,10 @@
         <v>93</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E16" s="18" t="str">
         <f>IF(C16=D16,"MATCH","MISMATCH")</f>
@@ -3826,10 +3826,10 @@
         <v>95</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E17" s="18" t="str">
         <f>IF(C17=D17,"MATCH","MISMATCH")</f>
@@ -3849,7 +3849,7 @@
         <v>144</v>
       </c>
       <c r="J17" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K17" s="5" t="str">
         <f>IF(E17="MISMATCH","STOP: ID number does not match the work list",IF(F17="Yes","STOP: error 56000, an endorsement is already in progress",IF(H17=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3876,10 +3876,10 @@
         <v>97</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E18" s="18" t="str">
         <f>IF(C18=D18,"MATCH","MISMATCH")</f>
@@ -3899,7 +3899,7 @@
         <v>144</v>
       </c>
       <c r="J18" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K18" s="5" t="str">
         <f>IF(E18="MISMATCH","STOP: ID number does not match the work list",IF(F18="Yes","STOP: error 56000, an endorsement is already in progress",IF(H18=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3926,10 +3926,10 @@
         <v>99</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E19" s="18" t="str">
         <f>IF(C19=D19,"MATCH","MISMATCH")</f>
@@ -3949,7 +3949,7 @@
         <v>144</v>
       </c>
       <c r="J19" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K19" s="5" t="str">
         <f>IF(E19="MISMATCH","STOP: ID number does not match the work list",IF(F19="Yes","STOP: error 56000, an endorsement is already in progress",IF(H19=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -3976,10 +3976,10 @@
         <v>102</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="E20" s="18" t="str">
         <f>IF(C20=D20,"MATCH","MISMATCH")</f>
@@ -4026,10 +4026,10 @@
         <v>104</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E21" s="18" t="str">
         <f>IF(C21=D21,"MATCH","MISMATCH")</f>
@@ -4076,20 +4076,20 @@
         <v>106</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E22" s="18" t="str">
         <f>IF(C22=D22,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G22" s="13" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H22" s="16">
         <f>INDEX('Fee Switch-Off'!$G$5:$G$30,MATCH($A22,'Fee Switch-Off'!$A$5:$A$30,0))</f>
@@ -4099,7 +4099,7 @@
         <v>144</v>
       </c>
       <c r="J22" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K22" s="5" t="str">
         <f>IF(E22="MISMATCH","STOP: ID number does not match the work list",IF(F22="Yes","STOP: error 56000, an endorsement is already in progress",IF(H22=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -4126,20 +4126,20 @@
         <v>109</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="E23" s="18" t="str">
         <f>IF(C23=D23,"MATCH","MISMATCH")</f>
         <v>MATCH</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G23" s="13" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H23" s="16">
         <f>INDEX('Fee Switch-Off'!$G$5:$G$30,MATCH($A23,'Fee Switch-Off'!$A$5:$A$30,0))</f>
@@ -4149,7 +4149,7 @@
         <v>144</v>
       </c>
       <c r="J23" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K23" s="5" t="str">
         <f>IF(E23="MISMATCH","STOP: ID number does not match the work list",IF(F23="Yes","STOP: error 56000, an endorsement is already in progress",IF(H23=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -4176,10 +4176,10 @@
         <v>112</v>
       </c>
       <c r="C24" s="22" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D24" s="22" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E24" s="18" t="str">
         <f>IF(C24=D24,"MATCH","MISMATCH")</f>
@@ -4199,7 +4199,7 @@
         <v>144</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K24" s="5" t="str">
         <f>IF(E24="MISMATCH","STOP: ID number does not match the work list",IF(F24="Yes","STOP: error 56000, an endorsement is already in progress",IF(H24=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -4226,10 +4226,10 @@
         <v>115</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E25" s="18" t="str">
         <f>IF(C25=D25,"MATCH","MISMATCH")</f>
@@ -4246,7 +4246,7 @@
         <v>0.575</v>
       </c>
       <c r="I25" s="23" t="s">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="J25" s="23" t="s">
         <v>36</v>
@@ -4296,7 +4296,7 @@
         <v>1.15</v>
       </c>
       <c r="I26" s="23" t="s">
-        <v>173</v>
+        <v>148</v>
       </c>
       <c r="J26" s="23" t="s">
         <v>146</v>
@@ -4349,7 +4349,7 @@
         <v>144</v>
       </c>
       <c r="J27" s="23" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K27" s="5" t="str">
         <f>IF(E27="MISMATCH","STOP: ID number does not match the work list",IF(F27="Yes","STOP: error 56000, an endorsement is already in progress",IF(H27=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -4399,7 +4399,7 @@
         <v>144</v>
       </c>
       <c r="J28" s="23" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="K28" s="5" t="str">
         <f>IF(E28="MISMATCH","STOP: ID number does not match the work list",IF(F28="Yes","STOP: error 56000, an endorsement is already in progress",IF(H28=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>
@@ -4449,7 +4449,7 @@
         <v>144</v>
       </c>
       <c r="J29" s="23" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K29" s="5" t="str">
         <f>IF(E29="MISMATCH","STOP: ID number does not match the work list",IF(F29="Yes","STOP: error 56000, an endorsement is already in progress",IF(H29=0,"SKIP: fee already 0.000","PROCEED: set VAT Inclusive fee to 0")))</f>

</xml_diff>